<commit_message>
feat(sprint-2): implement atmospheric thermodynamics, Dalton's partial pressures, and chemical equilibrium
</commit_message>
<xml_diff>
--- a/Terra_Colony_Simulator.xlsx
+++ b/Terra_Colony_Simulator.xlsx
@@ -1761,293 +1761,20 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="UTF-8" standalone="yes"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetFormatPr defaultRowHeight="18"/>
-  <cols>
-    <col min="1" max="1" width="26"/>
-    <col min="2" max="2" width="18"/>
-    <col min="3" max="3" width="16"/>
-    <col min="4" max="4" width="20"/>
-    <col min="5" max="5" width="38"/>
-    <col min="6" max="6" width="22"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="28">
-      <c r="A1" t="inlineStr" s="5">
-        <is>
-          <t>TERRA // ATMOSPHERIC TELEMETRY &amp; PLANETARY MODELS</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr" s="2">
-        <is>
-          <t>PARAMETER</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr" s="2">
-        <is>
-          <t>CURRENT VALUE</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr" s="2">
-        <is>
-          <t>UNIT</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr" s="2">
-        <is>
-          <t>TARGET RANGE</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr" s="2">
-        <is>
-          <t>STATUS / FORMULA</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr" s="2">
-        <is>
-          <t>HABITABILITY WEIGHT</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr" s="6">
-        <is>
-          <t>Surface Temperature</t>
-        </is>
-      </c>
-      <c r="B3" s="4">
-        <v>-65.0</v>
-      </c>
-      <c r="C3" t="inlineStr" s="4">
-        <is>
-          <t>°C</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr" s="4">
-        <is>
-          <t>+14.0 to +18.0</t>
-        </is>
-      </c>
-      <c r="E3" s="4">
-        <f>=-65.0 + (B4*0.04) + 2.5</f>
-      </c>
-      <c r="F3" t="inlineStr" s="4">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr" s="6">
-        <is>
-          <t>Atmospheric Pressure</t>
-        </is>
-      </c>
-      <c r="B4" s="4">
-        <v>180.0</v>
-      </c>
-      <c r="C4" t="inlineStr" s="4">
-        <is>
-          <t>hPa</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr" s="4">
-        <is>
-          <t>980.0 to 1025.0</t>
-        </is>
-      </c>
-      <c r="E4" s="4">
-        <f>=180 + SUM(B9:B12)</f>
-      </c>
-      <c r="F4" t="inlineStr" s="4">
-        <is>
-          <t>25%</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr" s="6">
-        <is>
-          <t>Atmospheric Oxygen</t>
-        </is>
-      </c>
-      <c r="B5" s="4">
-        <v>0.1</v>
-      </c>
-      <c r="C5" t="inlineStr" s="4">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr" s="4">
-        <is>
-          <t>19.5% to 21.5%</t>
-        </is>
-      </c>
-      <c r="E5" s="4">
-        <f>=0.1 + (COUNTIF(Surface_Sector_Grid!B5:Q20, "*AG*") * 0.35)</f>
-      </c>
-      <c r="F5" t="inlineStr" s="4">
-        <is>
-          <t>30%</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr" s="6">
-        <is>
-          <t>Hydrosphere Volume</t>
-        </is>
-      </c>
-      <c r="B6" s="4">
-        <v>65.0</v>
-      </c>
-      <c r="C6" t="inlineStr" s="4">
-        <is>
-          <t>Mega-Liters</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr" s="4">
-        <is>
-          <t>800.0 to 1500.0</t>
-        </is>
-      </c>
-      <c r="E6" s="4">
-        <f>=65.0 + IF(B3&gt;0, (B3*12), 0)</f>
-      </c>
-      <c r="F6" t="inlineStr" s="4">
-        <is>
-          <t>20%</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr" s="1">
-        <is>
-          <t>HABITABILITY INDEX</t>
-        </is>
-      </c>
-      <c r="B7" s="1">
-        <v>4.2</v>
-      </c>
-      <c r="C7" t="inlineStr" s="1">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr" s="1">
-        <is>
-          <t>100.0%</t>
-        </is>
-      </c>
-      <c r="E7" s="1">
-        <f>=ROUND(IF(B3&gt;-10,25,0)+IF(B4&gt;800,25,0)+IF(B5&gt;18,30,0)+IF(B6&gt;600,20,0),1)</f>
-      </c>
-      <c r="F7" t="inlineStr" s="1">
-        <is>
-          <t>OVERALL</t>
-        </is>
-      </c>
-    </row>
-    <row r="8"/>
-    <row r="9">
-      <c r="A9" t="inlineStr" s="2">
-        <is>
-          <t>GAS COMPOSITION INVENTORY</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr" s="2">
-        <is>
-          <t>PARTIAL PRESSURE (hPa)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr" s="2">
-        <is>
-          <t>RATIO (%)</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr" s="2">
-        <is>
-          <t>PRIMARY SOURCE</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr" s="0">
-        <is>
-          <t>Carbon Dioxide (CO2)</t>
-        </is>
-      </c>
-      <c r="B10" s="0">
-        <v>170.0</v>
-      </c>
-      <c r="C10" s="0">
-        <v>94.4</v>
-      </c>
-      <c r="D10" t="inlineStr" s="0">
-        <is>
-          <t>Native Martian Basin</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr" s="0">
-        <is>
-          <t>Nitrogen Buffer (N2)</t>
-        </is>
-      </c>
-      <c r="B11" s="0">
-        <v>8.5</v>
-      </c>
-      <c r="C11" s="0">
-        <v>4.7</v>
-      </c>
-      <c r="D11" t="inlineStr" s="0">
-        <is>
-          <t>Atmospheric Scrubbers</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr" s="0">
-        <is>
-          <t>Oxygen Gas (O2)</t>
-        </is>
-      </c>
-      <c r="B12" s="0">
-        <v>0.18</v>
-      </c>
-      <c r="C12" s="0">
-        <v>0.1</v>
-      </c>
-      <c r="D12" t="inlineStr" s="0">
-        <is>
-          <t>Cyanobacteria Greenhouses</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr" s="0">
-        <is>
-          <t>Water Vapor (H2O)</t>
-        </is>
-      </c>
-      <c r="B13" s="0">
-        <v>1.32</v>
-      </c>
-      <c r="C13" s="0">
-        <v>0.8</v>
-      </c>
-      <c r="D13" t="inlineStr" s="0">
-        <is>
-          <t>Polar Ice Sublimation</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
+    <sheetFormatPr defaultRowHeight="18"/>
+    <cols>
+        <col min="1" max="1" width="26"/>
+        <col min="2" max="2" width="18"/>
+        <col min="3" max="3" width="16"/>
+        <col min="4" max="4" width="20"/>
+        <col min="5" max="5" width="38"/>
+        <col min="6" max="6" width="22"/>
+    </cols>
+    <sheetData>
+        <row r="1" ht="28"><c r="A1" t="inlineStr" s="5"><is><t>TERRA // ATMOSPHERIC TELEMETRY &amp; PLANETARY MODELS</t></is></c></row><row r="2"><c r="A2" t="inlineStr" s="2"><is><t>PARAMETER</t></is></c> <c r="B2" t="inlineStr" s="2"><is><t>CURRENT VALUE</t></is></c> <c r="C2" t="inlineStr" s="2"><is><t>UNIT</t></is></c> <c r="D2" t="inlineStr" s="2"><is><t>TARGET RANGE</t></is></c> <c r="E2" t="inlineStr" s="2"><is><t>STATUS / FORMULA</t></is></c> <c r="F2" t="inlineStr" s="2"><is><t>HABITABILITY WEIGHT</t></is></c></row><row r="3"><c r="A3" t="inlineStr" s="6"><is><t>Surface Temperature</t></is></c> <c r="B3" s="4"><v>-65.0</v></c> <c r="C3" t="inlineStr" s="4"><is><t>°C</t></is></c> <c r="D3" t="inlineStr" s="4"><is><t>+14.0 to +18.0</t></is></c> <c r="E3" s="4"><f>=-65.0 + (COUNTIF(Surface_Sector_Grid!B5:Q20, "*GD*") * 0.6) + (COUNTIF(Surface_Sector_Grid!B5:Q20, "*TF*") * 1.5) + (B10 * 0.05)</f></c> <c r="F3" t="inlineStr" s="4"><is><t>25%</t></is></c></row><row r="4"><c r="A4" t="inlineStr" s="6"><is><t>Atmospheric Pressure</t></is></c> <c r="B4" s="4"><v>180.0</v></c> <c r="C4" t="inlineStr" s="4"><is><t>hPa</t></is></c> <c r="D4" t="inlineStr" s="4"><is><t>980.0 to 1025.0</t></is></c> <c r="E4" s="4"><f>=180.0 + (COUNTIF(Surface_Sector_Grid!B5:Q20, "*TF*") * 12.0) + (COUNTIF(Surface_Sector_Grid!B5:Q20, "*AS*") * 15.0)</f></c> <c r="F4" t="inlineStr" s="4"><is><t>25%</t></is></c></row><row r="5"><c r="A5" t="inlineStr" s="6"><is><t>Atmospheric Oxygen</t></is></c> <c r="B5" s="4"><v>0.1</v></c> <c r="C5" t="inlineStr" s="4"><is><t>%</t></is></c> <c r="D5" t="inlineStr" s="4"><is><t>19.5% to 21.5%</t></is></c> <c r="E5" s="4"><f>=0.10 + (COUNTIF(Surface_Sector_Grid!B5:Q20, "*AG*") * 0.35) + (COUNTIF(Surface_Sector_Grid!B5:Q20, "♣♣") * 0.05)</f></c> <c r="F5" t="inlineStr" s="4"><is><t>30%</t></is></c></row><row r="6"><c r="A6" t="inlineStr" s="6"><is><t>Hydrosphere Volume</t></is></c> <c r="B6" s="4"><v>65.0</v></c> <c r="C6" t="inlineStr" s="4"><is><t>Mega-Liters</t></is></c> <c r="D6" t="inlineStr" s="4"><is><t>800.0 to 1500.0</t></is></c> <c r="E6" s="4"><f>=65.0 + (COUNTIF(Surface_Sector_Grid!B5:Q20, "*IH*") * 25.0) + IF(B3 > 0, (COUNTIF(Surface_Sector_Grid!B5:Q20, "≈≈") * 10.0), 0)</f></c> <c r="F6" t="inlineStr" s="4"><is><t>20%</t></is></c></row><row r="7"><c r="A7" t="inlineStr" s="1"><is><t>HABITABILITY INDEX</t></is></c> <c r="B7" s="1"><v>4.2</v></c> <c r="C7" t="inlineStr" s="1"><is><t>%</t></is></c> <c r="D7" t="inlineStr" s="1"><is><t>100.0%</t></is></c> <c r="E7" s="1"><f>=MIN(100, ROUND(IF(AND(B3>=-10, B3<=30), 25, MAX(0, 25 - ABS(B3-15)*0.5)) + IF(B4>=800, 25, 25*(B4/1000)) + IF(B5>=18, 30, 30*(B5/20)) + IF(B6>=500, 20, 20*(B6/500)), 1))</f></c> <c r="F7" t="inlineStr" s="1"><is><t>OVERALL</t></is></c></row><row r="8"/><row r="9"><c r="A9" t="inlineStr" s="2"><is><t>GAS COMPOSITION INVENTORY</t></is></c> <c r="B9" t="inlineStr" s="2"><is><t>PARTIAL PRESSURE (hPa)</t></is></c> <c r="C9" t="inlineStr" s="2"><is><t>RATIO (%)</t></is></c> <c r="D9" t="inlineStr" s="2"><is><t>PRIMARY SOURCE</t></is></c></row><row r="10"><c r="A10" t="inlineStr" s="0"><is><t>Carbon Dioxide (CO2)</t></is></c> <c r="B10" s="4"><f>=MAX(0, B4 - B11 - B12 - B13)</f></c> <c r="C10" s="4"><f>=ROUND(B10/B$4*100, 1)</f></c> <c r="D10" t="inlineStr" s="0"><is><t>Native Martian Basin &amp; Gas Factories</t></is></c></row><row r="11"><c r="A11" t="inlineStr" s="0"><is><t>Nitrogen Buffer (N2)</t></is></c> <c r="B11" s="4"><f>=8.5 + (COUNTIF(Surface_Sector_Grid!B5:Q20, "*AS*") * 15.0)</f></c> <c r="C11" s="4"><f>=ROUND(B11/B$4*100, 1)</f></c> <c r="D11" t="inlineStr" s="0"><is><t>Atmospheric Scrubbers</t></is></c></row><row r="12"><c r="A12" t="inlineStr" s="0"><is><t>Oxygen Gas (O2)</t></is></c> <c r="B12" s="4"><f>=ROUND(B4 * (B5 / 100), 2)</f></c> <c r="C12" s="4"><f>=ROUND(B12/B$4*100, 1)</f></c> <c r="D12" t="inlineStr" s="0"><is><t>Cyanobacteria Greenhouses &amp; Biomes</t></is></c></row><row r="13"><c r="A13" t="inlineStr" s="0"><is><t>Water Vapor (H2O)</t></is></c> <c r="B13" s="4"><f>=ROUND(1.32 + IF(B3 > 0, B3 * 0.35, 0), 2)</f></c> <c r="C13" s="4"><f>=ROUND(B13/B$4*100, 1)</f></c> <c r="D13" t="inlineStr" s="0"><is><t>Polar Ice Sublimation &amp; Ocean Thaw</t></is></c></row>
+    </sheetData>
 </worksheet>
 </file>
 

</xml_diff>